<commit_message>
feat: ticket analysis V2, pain point clustering, and insight overview upgrades.
Add ticketAnalysis pipeline (customer request, pain point, optimization), V2 pain clustering with journey/overview integration, customer tier import, snapshot rehydration for legacy recommendations, expanded tests and docs, plus storage and taxonomy/config updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/config/taxonomy/打标配置.xlsx
+++ b/public/config/taxonomy/打标配置.xlsx
@@ -4,12 +4,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="填写说明" sheetId="1" r:id="rId1"/>
-    <sheet name="请求节点-服务类型" sheetId="2" r:id="rId2"/>
-    <sheet name="请求节点-问题子类" sheetId="3" r:id="rId3"/>
-    <sheet name="产品识别" sheetId="4" r:id="rId4"/>
-    <sheet name="用户旅程" sheetId="5" r:id="rId5"/>
-    <sheet name="请求场景" sheetId="6" r:id="rId6"/>
-    <sheet name="通用问题类型" sheetId="7" r:id="rId7"/>
+    <sheet name="产品识别" sheetId="2" r:id="rId2"/>
+    <sheet name="用户旅程" sheetId="3" r:id="rId3"/>
+    <sheet name="通用问题类型" sheetId="4" r:id="rId4"/>
+    <sheet name="请求节点-服务类型" sheetId="5" r:id="rId5"/>
+    <sheet name="请求节点-问题子类" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -38,11 +37,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="5">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
   </numFmts>
   <fonts count="1">
@@ -448,7 +443,7 @@
         <v>产品Key、产品名称、匹配关键词（逗号分隔）</v>
       </c>
       <c r="D3" t="str">
-        <v>eip | 弹性公网 IP | 弹性公网,公网IP,EIP</v>
+        <v>vpc | 虚拟私有云 | 虚拟私有云,VPC,vpc,专有网络</v>
       </c>
     </row>
     <row r="4">
@@ -462,7 +457,7 @@
         <v>一级/二级 ID·名称·说明、参考关键词。旅程打标与主题标签均只维护本表（必填）</v>
       </c>
       <c r="D4" t="str">
-        <v>eip | bind | 绑定与网络配置 | … | bind-resource | 绑定/解绑云资源 | …</v>
+        <v>vpc | provision | 资源申请与开通 | … | create-vpc | 创建VPC与子网 | …</v>
       </c>
     </row>
     <row r="5">
@@ -473,10 +468,10 @@
         <v>全平台共用</v>
       </c>
       <c r="C5" t="str">
-        <v>无产品Key。问题类型名称、说明、参考关键词</v>
+        <v>无产品Key。问题类型名称、说明、参考关键词（12 类，与决策树 classifier 一致）</v>
       </c>
       <c r="D5" t="str">
-        <v>可用性/连通性 | 连通、中断类问题 | 不通,无法访问</v>
+        <v>可用性/连通性故障 | 业务完全中断、网络不通 | 不通,无法访问,中断</v>
       </c>
     </row>
     <row r="6">
@@ -564,7 +559,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
@@ -573,20 +567,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:C6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>产品Key</v>
       </c>
       <c r="B1" t="str">
-        <v>请求节点服务类型</v>
+        <v>产品名称</v>
       </c>
       <c r="C1" t="str">
-        <v>一级ID</v>
-      </c>
-      <c r="D1" t="str">
-        <v>一级名称</v>
+        <v>匹配关键词</v>
       </c>
     </row>
     <row r="2">
@@ -594,101 +585,91 @@
         <v>eip</v>
       </c>
       <c r="B2" t="str">
-        <v>产品咨询</v>
+        <v>弹性公网IP</v>
       </c>
       <c r="C2" t="str">
-        <v>discover</v>
-      </c>
-      <c r="D2" t="str">
-        <v>认知与选型</v>
+        <v>弹性公网IP,eip</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>eip</v>
+        <v>generic</v>
       </c>
       <c r="B3" t="str">
-        <v>产品使用问题</v>
+        <v>通用产品</v>
       </c>
       <c r="C3" t="str">
-        <v>operate</v>
-      </c>
-      <c r="D3" t="str">
-        <v>业务使用与连通</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>eip</v>
+        <v>dc</v>
       </c>
       <c r="B4" t="str">
-        <v>产品功能</v>
+        <v>云专线</v>
       </c>
       <c r="C4" t="str">
-        <v>discover</v>
-      </c>
-      <c r="D4" t="str">
-        <v>认知与选型</v>
+        <v>云专线,ecc,dc,专线,跨省专线,MPLS,云互联,CENO-SL,CENO-NET,MOP-T,MOP-O,云网一体,客响,勘察单,移机工单,汇聚专线,用户侧子网,互联地址</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>eip</v>
+        <v>slb</v>
       </c>
       <c r="B5" t="str">
-        <v>产品使用</v>
+        <v>弹性负载均衡</v>
       </c>
       <c r="C5" t="str">
-        <v>operate</v>
-      </c>
-      <c r="D5" t="str">
-        <v>业务使用与连通</v>
+        <v>弹性负载均衡,SLB,slb,负载均衡,ELB,应用型负载均衡,网络型负载均衡</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>eip</v>
+        <v>vpc</v>
       </c>
       <c r="B6" t="str">
-        <v>其他</v>
+        <v>虚拟私有云</v>
       </c>
       <c r="C6" t="str">
-        <v>service</v>
-      </c>
-      <c r="D6" t="str">
-        <v>服务与体验</v>
+        <v>虚拟私有云,VPC,vpc,专有网络,私有网络</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:H105"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>产品Key</v>
       </c>
       <c r="B1" t="str">
-        <v>请求节点问题子类</v>
+        <v>一级ID</v>
       </c>
       <c r="C1" t="str">
-        <v>一级ID</v>
+        <v>一级名称</v>
       </c>
       <c r="D1" t="str">
-        <v>一级名称</v>
+        <v>一级说明</v>
       </c>
       <c r="E1" t="str">
         <v>二级ID</v>
       </c>
       <c r="F1" t="str">
         <v>二级名称</v>
+      </c>
+      <c r="G1" t="str">
+        <v>二级说明</v>
+      </c>
+      <c r="H1" t="str">
+        <v>参考关键词</v>
       </c>
     </row>
     <row r="2">
@@ -696,19 +677,25 @@
         <v>eip</v>
       </c>
       <c r="B2" t="str">
-        <v>IP无法访问</v>
+        <v>discover</v>
       </c>
       <c r="C2" t="str">
-        <v>operate</v>
+        <v>认知与选型</v>
       </c>
       <c r="D2" t="str">
-        <v>业务使用与连通</v>
+        <v>客户了解弹性公网 IP 是什么、适用场景、与固定公网/共享带宽的区别，咨询规格、线路类型（BGP/单线）、IPv4/IPv6 及资费模型</v>
       </c>
       <c r="E2" t="str">
-        <v>operate-access</v>
+        <v>discover-intro</v>
       </c>
       <c r="F2" t="str">
-        <v>公网访问不通</v>
+        <v>产品与规格咨询</v>
+      </c>
+      <c r="G2" t="str">
+        <v>产品能力介绍、计费项说明、带宽规格选择、是否支持 IPv6、与竞品对比</v>
+      </c>
+      <c r="H2" t="str">
+        <v>产品咨询,了解,选型,规格,资费,IPv6,BGP,产品介绍</v>
       </c>
     </row>
     <row r="3">
@@ -716,216 +703,6 @@
         <v>eip</v>
       </c>
       <c r="B3" t="str">
-        <v>产品功能</v>
-      </c>
-      <c r="C3" t="str">
-        <v>discover</v>
-      </c>
-      <c r="D3" t="str">
-        <v>认知与选型</v>
-      </c>
-      <c r="E3" t="str">
-        <v>discover-intro</v>
-      </c>
-      <c r="F3" t="str">
-        <v>产品与规格咨询</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>eip</v>
-      </c>
-      <c r="B4" t="str">
-        <v>产品咨询</v>
-      </c>
-      <c r="C4" t="str">
-        <v>discover</v>
-      </c>
-      <c r="D4" t="str">
-        <v>认知与选型</v>
-      </c>
-      <c r="E4" t="str">
-        <v>discover-intro</v>
-      </c>
-      <c r="F4" t="str">
-        <v>产品与规格咨询</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>eip</v>
-      </c>
-      <c r="B5" t="str">
-        <v>其他</v>
-      </c>
-      <c r="C5" t="str">
-        <v>operate</v>
-      </c>
-      <c r="D5" t="str">
-        <v>业务使用与连通</v>
-      </c>
-      <c r="E5" t="str">
-        <v>operate-quality</v>
-      </c>
-      <c r="F5" t="str">
-        <v>网络质量与丢包</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>eip</v>
-      </c>
-      <c r="B6" t="str">
-        <v>公网IP绑定/解绑失败</v>
-      </c>
-      <c r="C6" t="str">
-        <v>bind</v>
-      </c>
-      <c r="D6" t="str">
-        <v>绑定与网络配置</v>
-      </c>
-      <c r="E6" t="str">
-        <v>bind-resource</v>
-      </c>
-      <c r="F6" t="str">
-        <v>绑定/解绑云资源</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>产品Key</v>
-      </c>
-      <c r="B1" t="str">
-        <v>产品名称</v>
-      </c>
-      <c r="C1" t="str">
-        <v>匹配关键词</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>eip</v>
-      </c>
-      <c r="B2" t="str">
-        <v>弹性公网IP</v>
-      </c>
-      <c r="C2" t="str">
-        <v>弹性公网IP,eip</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>generic</v>
-      </c>
-      <c r="B3" t="str">
-        <v>通用产品</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>dc</v>
-      </c>
-      <c r="B4" t="str">
-        <v>云专线</v>
-      </c>
-      <c r="C4" t="str">
-        <v>云专线,ecc,dc,专线,跨省专线,MPLS,云互联,CENO-SL,CENO-NET,MOP-T,MOP-O,云网一体,客响,勘察单,移机工单,汇聚专线,用户侧子网,互联地址</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>slb</v>
-      </c>
-      <c r="B5" t="str">
-        <v>弹性负载均衡</v>
-      </c>
-      <c r="C5" t="str">
-        <v>弹性负载均衡,SLB,slb,负载均衡,ELB,应用型负载均衡,网络型负载均衡</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H78"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>产品Key</v>
-      </c>
-      <c r="B1" t="str">
-        <v>一级ID</v>
-      </c>
-      <c r="C1" t="str">
-        <v>一级名称</v>
-      </c>
-      <c r="D1" t="str">
-        <v>一级说明</v>
-      </c>
-      <c r="E1" t="str">
-        <v>二级ID</v>
-      </c>
-      <c r="F1" t="str">
-        <v>二级名称</v>
-      </c>
-      <c r="G1" t="str">
-        <v>二级说明</v>
-      </c>
-      <c r="H1" t="str">
-        <v>参考关键词</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>eip</v>
-      </c>
-      <c r="B2" t="str">
-        <v>discover</v>
-      </c>
-      <c r="C2" t="str">
-        <v>认知与选型</v>
-      </c>
-      <c r="D2" t="str">
-        <v>客户了解弹性公网 IP 是什么、适用场景、与固定公网/共享带宽的区别，咨询规格、线路类型（BGP/单线）、IPv4/IPv6 及资费模型</v>
-      </c>
-      <c r="E2" t="str">
-        <v>discover-intro</v>
-      </c>
-      <c r="F2" t="str">
-        <v>产品与规格咨询</v>
-      </c>
-      <c r="G2" t="str">
-        <v>产品能力介绍、计费项说明、带宽规格选择、是否支持 IPv6、与竞品对比</v>
-      </c>
-      <c r="H2" t="str">
-        <v>产品咨询，了解，选型，规格，资费，IPv6，BGP，产品介绍</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>eip</v>
-      </c>
-      <c r="B3" t="str">
         <v>discover</v>
       </c>
       <c r="C3" t="str">
@@ -944,7 +721,7 @@
         <v>按带宽/按流量、包年包月、共享带宽、折扣券、账单项解释</v>
       </c>
       <c r="H3" t="str">
-        <v>计费，折扣，账单，按量，包年，共享带宽，扣费规则</v>
+        <v>计费,折扣,账单,按量,包年,共享带宽,扣费规则</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -981,7 +758,7 @@
 账号信息不完整</v>
       </c>
       <c r="H4" t="str">
-        <v>创建，开通，申购，订购，申请，新建，购买</v>
+        <v>创建,开通,申购,订购,申请,新建,购买</v>
       </c>
     </row>
     <row r="5">
@@ -1007,7 +784,7 @@
         <v>调整公网带宽、限速、带宽包、订单无法操作、升配降配失败</v>
       </c>
       <c r="H5" t="str">
-        <v>带宽，升降配，调整带宽，限速，扩容，降配，订单无法操作</v>
+        <v>带宽,升降配,调整带宽,限速,扩容,降配,订单无法操作</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -1073,7 +850,7 @@
 剩余配额被冻结</v>
       </c>
       <c r="H7" t="str">
-        <v>配额，权限，无法创建，开通失败，系统错误，订单失败</v>
+        <v>配额,权限,无法创建,开通失败,系统错误,订单失败</v>
       </c>
     </row>
     <row r="8">
@@ -1256,7 +1033,7 @@
         <v>EIP 移入、移出共享带宽失败</v>
       </c>
       <c r="H14" t="str">
-        <v>绑定，解绑，挂载，关联，云主机，ECS，网卡，ENI，绑定失败，空闲</v>
+        <v>绑定,解绑,挂载,关联,云主机,ECS,网卡,ENI,绑定失败,空闲</v>
       </c>
     </row>
     <row r="15">
@@ -1360,7 +1137,7 @@
         <v>安全组、端口开放、白名单、ACL、仅允许特定 IP 访问</v>
       </c>
       <c r="H18" t="str">
-        <v>白名单，安全组，端口，ACL，开放，8085，防火墙</v>
+        <v>白名单,安全组,端口,ACL,开放,8085,防火墙</v>
       </c>
     </row>
     <row r="19" xml:space="preserve">
@@ -1420,7 +1197,7 @@
 非移动云IP</v>
       </c>
       <c r="H19" t="str">
-        <v>无法访问，不通，外网，百度，IP无法访问，访问不了，连不上，远程，登录，SSH，RDP，3389，远程连接，远程登录，丢包，波动，延迟，不稳定，PING，卡顿，质量，网络波动</v>
+        <v>无法访问,不通,外网,百度,IP无法访问,访问不了,连不上,远程,登录,SSH,RDP,3389,远程连接,远程登录,丢包,波动,延迟,不稳定,PING,卡顿,质量,网络波动</v>
       </c>
     </row>
     <row r="20">
@@ -1446,7 +1223,7 @@
         <v>流量查询、监控数据、某时段流量核实、计费流量争议</v>
       </c>
       <c r="H20" t="str">
-        <v>流量，监控，查询流量，时段，流量是否，统计</v>
+        <v>流量,监控,查询流量,时段,流量是否,统计</v>
       </c>
     </row>
     <row r="21">
@@ -1472,7 +1249,7 @@
         <v>业务中断、大面积不可用、影响客户业务、故障时段明确</v>
       </c>
       <c r="H21" t="str">
-        <v>中断，业务影响，不可用，宕机，故障，应急</v>
+        <v>中断,业务影响,不可用,宕机,故障,应急</v>
       </c>
     </row>
     <row r="22">
@@ -1524,7 +1301,7 @@
         <v>退订 EIP、释放公网 IP、到期删除、注销，</v>
       </c>
       <c r="H23" t="str">
-        <v>退订，释放，删除，注销，到期</v>
+        <v>退订,释放,删除,注销,到期</v>
       </c>
     </row>
     <row r="24" xml:space="preserve">
@@ -1560,7 +1337,7 @@
 客户对订购规则不了解</v>
       </c>
       <c r="H24" t="str">
-        <v>无法退订，退订失败，无法删除，协助删除，内部系统错误</v>
+        <v>无法退订,退订失败,无法删除,协助删除,内部系统错误</v>
       </c>
     </row>
     <row r="25">
@@ -1638,7 +1415,7 @@
         <v>服务态度、响应慢、回访要求、升级投诉</v>
       </c>
       <c r="H27" t="str">
-        <v>投诉，客服，态度，回访，金牌，不满</v>
+        <v>投诉,客服,态度,回访,金牌,不满</v>
       </c>
     </row>
     <row r="28">
@@ -1664,7 +1441,7 @@
         <v>工单流转慢、跨部门协同、OP/后台处理时效</v>
       </c>
       <c r="H28" t="str">
-        <v>流转，协同，催单，处理慢，等待</v>
+        <v>流转,协同,催单,处理慢,等待</v>
       </c>
     </row>
     <row r="29">
@@ -1690,7 +1467,7 @@
         <v>一般咨询</v>
       </c>
       <c r="H29" t="str">
-        <v>咨询，了解</v>
+        <v>咨询,了解</v>
       </c>
     </row>
     <row r="30">
@@ -1716,7 +1493,7 @@
         <v>开通与配置</v>
       </c>
       <c r="H30" t="str">
-        <v>开通，配置</v>
+        <v>开通,配置</v>
       </c>
     </row>
     <row r="31">
@@ -1742,7 +1519,7 @@
         <v>日常运维</v>
       </c>
       <c r="H31" t="str">
-        <v>使用，运维</v>
+        <v>使用,运维</v>
       </c>
     </row>
     <row r="32">
@@ -1768,7 +1545,7 @@
         <v>故障处理</v>
       </c>
       <c r="H32" t="str">
-        <v>故障，排查</v>
+        <v>故障,排查</v>
       </c>
     </row>
     <row r="33">
@@ -1794,7 +1571,7 @@
         <v>带宽改配费用、折扣、官网价格、事业部折扣等</v>
       </c>
       <c r="H33" t="str">
-        <v>资费，价格，费用，多少钱，原价，折扣，一键折扣，集团折扣，官网查不到价格，数智事业部</v>
+        <v>资费,价格,费用,多少钱,原价,折扣,一键折扣,集团折扣,官网查不到价格,数智事业部</v>
       </c>
     </row>
     <row r="34">
@@ -1820,7 +1597,7 @@
         <v>跨账号拉线、备份速率、是否支持某能力等方案咨询</v>
       </c>
       <c r="H34" t="str">
-        <v>咨询，方案，是否支持，能不能，同时拉两条，上传速率，100M带宽，对象存储，备份软件</v>
+        <v>咨询,方案,是否支持,能不能,同时拉两条,上传速率,100M带宽,对象存储,备份软件</v>
       </c>
     </row>
     <row r="35">
@@ -1846,7 +1623,7 @@
         <v>开通、订购、审批、安装交付、汇聚专线权限</v>
       </c>
       <c r="H35" t="str">
-        <v>开通，订购，申购，加急，尽快开通，业务开通审批，安装交付，汇聚专线，订购权限</v>
+        <v>开通,订购,申购,加急,尽快开通,业务开通审批,安装交付,汇聚专线,订购权限</v>
       </c>
     </row>
     <row r="36">
@@ -1872,7 +1649,7 @@
         <v>开通失败但资源可用、未出账、MOP 订单状态</v>
       </c>
       <c r="H36" t="str">
-        <v>开通失败，订单状态，未出账，MOP-T，MOP-O，EMOP，资源可用，订单编号</v>
+        <v>开通失败,订单状态,未出账,MOP-T,MOP-O,EMOP,资源可用,订单编号</v>
       </c>
     </row>
     <row r="37">
@@ -1898,7 +1675,7 @@
         <v>可用区选择、VPC 子网无法选择、资源池限制</v>
       </c>
       <c r="H37" t="str">
-        <v>资源池，可用区，AZ，可用区2，可用区4，华东，苏州，郑州，选不了，VPC子网无法选择</v>
+        <v>资源池,可用区,AZ,可用区2,可用区4,华东,苏州,郑州,选不了,VPC子网无法选择</v>
       </c>
     </row>
     <row r="38">
@@ -1924,7 +1701,7 @@
         <v>跨省专线、当地客响、落地机房端口</v>
       </c>
       <c r="H38" t="str">
-        <v>跨省，青岛，医保，当地，客响，落地，机房，端口开放，地市</v>
+        <v>跨省,青岛,医保,当地,客响,落地,机房,端口开放,地市</v>
       </c>
     </row>
     <row r="39">
@@ -1950,7 +1727,7 @@
         <v>用户侧子网、白名单、子网冲突、VPC 变更</v>
       </c>
       <c r="H39" t="str">
-        <v>子网，用户侧子网，白名单，子网冲突，VPC变更，添加子网，网段冲突</v>
+        <v>子网,用户侧子网,白名单,子网冲突,VPC变更,添加子网,网段冲突</v>
       </c>
     </row>
     <row r="40">
@@ -1976,7 +1753,7 @@
         <v>路由策略、默认互联地址、dummy IP、边界网关</v>
       </c>
       <c r="H40" t="str">
-        <v>路由，路由策略，互联地址，默认互联，dummy，边界网关，tracert，网关地址</v>
+        <v>路由,路由策略,互联地址,默认互联,dummy,边界网关,tracert,网关地址</v>
       </c>
     </row>
     <row r="41">
@@ -2002,7 +1779,7 @@
         <v>跨账号/跨账户专线、同 VPC 子网、跨资源池路由</v>
       </c>
       <c r="H41" t="str">
-        <v>跨账号，跨账户，VPC，跨资源池，同一vpc，用户子网相同，云防火墙，路由规则</v>
+        <v>跨账号,跨账户,VPC,跨资源池,同一vpc,用户子网相同,云防火墙,路由规则</v>
       </c>
     </row>
     <row r="42">
@@ -2028,7 +1805,7 @@
         <v>不通、无法访问、ping 不通、访问云主机失败</v>
       </c>
       <c r="H42" t="str">
-        <v>不通，无法访问，ping不通，无法ping，连不上，无法连通，经常不通，访问云主机</v>
+        <v>不通,无法访问,ping不通,无法ping,连不上,无法连通,经常不通,访问云主机</v>
       </c>
     </row>
     <row r="43">
@@ -2054,7 +1831,7 @@
         <v>比公网慢、HIS 卡顿、上下行不对等</v>
       </c>
       <c r="H43" t="str">
-        <v>慢，速度慢，反应慢，卡顿，比公网慢，不对等，延迟差，HIS，加载慢</v>
+        <v>慢,速度慢,反应慢,卡顿,比公网慢,不对等,延迟差,HIS,加载慢</v>
       </c>
     </row>
     <row r="44">
@@ -2080,7 +1857,7 @@
         <v>丢包、波动、抖动、跨省链路质量</v>
       </c>
       <c r="H44" t="str">
-        <v>丢包，跨省链路，波动，抖动，链路质量，质量差</v>
+        <v>丢包,跨省链路,波动,抖动,链路质量,质量差</v>
       </c>
     </row>
     <row r="45">
@@ -2106,7 +1883,7 @@
         <v>带宽超限、流量监控、利用率查询</v>
       </c>
       <c r="H45" t="str">
-        <v>带宽超限，监控，流量，利用率，超限情况</v>
+        <v>带宽超限,监控,流量,利用率,超限情况</v>
       </c>
     </row>
     <row r="46">
@@ -2132,7 +1909,7 @@
         <v>扩容升配、500M改5G、带宽不足无法扩容</v>
       </c>
       <c r="H46" t="str">
-        <v>带宽变更，扩容，升配，500M，5G，提速，变更带宽，带宽不足，无法扩容</v>
+        <v>带宽变更,扩容,升配,500M,5G,提速,变更带宽,带宽不足,无法扩容</v>
       </c>
     </row>
     <row r="47">
@@ -2158,7 +1935,7 @@
         <v>移机工单、勘察、割接保障、CNSO</v>
       </c>
       <c r="H47" t="str">
-        <v>移机，搬迁，割接，移机工单，勘察，CNSO，云网一体，节点流程，割接保障</v>
+        <v>移机,搬迁,割接,移机工单,勘察,CNSO,云网一体,节点流程,割接保障</v>
       </c>
     </row>
     <row r="48">
@@ -2184,7 +1961,7 @@
         <v>资源池迁移、两条专线并存、退订旧线</v>
       </c>
       <c r="H48" t="str">
-        <v>迁移，业务迁移，两条专线，同时存在，退订杭州，资源池迁移</v>
+        <v>迁移,业务迁移,两条专线,同时存在,退订杭州,资源池迁移</v>
       </c>
     </row>
     <row r="49">
@@ -2210,7 +1987,7 @@
         <v>中断、大面积不可用、应急</v>
       </c>
       <c r="H49" t="str">
-        <v>中断，业务影响，不可用，大面积，应急</v>
+        <v>中断,业务影响,不可用,大面积,应急</v>
       </c>
     </row>
     <row r="50">
@@ -2236,7 +2013,7 @@
         <v>协查、后台核实、抓包定位</v>
       </c>
       <c r="H50" t="str">
-        <v>协查，排查，根因，抓包，协助核实，后台，定位</v>
+        <v>协查,排查,根因,抓包,协助核实,后台,定位</v>
       </c>
     </row>
     <row r="51">
@@ -2262,7 +2039,7 @@
         <v>退订、撤销订单、欠费恢复</v>
       </c>
       <c r="H51" t="str">
-        <v>退订，撤销，欠费，恢复数据，被退订，冲突订单</v>
+        <v>退订,撤销,欠费,恢复数据,被退订,冲突订单</v>
       </c>
     </row>
     <row r="52">
@@ -2288,7 +2065,7 @@
         <v>专线暂停恢复、续订按钮</v>
       </c>
       <c r="H52" t="str">
-        <v>暂停，恢复，续订，续费，续订按钮，跨账号实例</v>
+        <v>暂停,恢复,续订,续费,续订按钮,跨账号实例</v>
       </c>
     </row>
     <row r="53">
@@ -2314,7 +2091,7 @@
         <v>计费清单、出账规则、冲销计算、加急要清单</v>
       </c>
       <c r="H53" t="str">
-        <v>账单，计费清单，出账，如何计算，冲销，1月到3月，清单，加急要清单</v>
+        <v>账单,计费清单,出账,如何计算,冲销,1月到3月,清单,加急要清单</v>
       </c>
     </row>
     <row r="54">
@@ -2340,7 +2117,7 @@
         <v>催进度、环节审批、省内传输开通</v>
       </c>
       <c r="H54" t="str">
-        <v>催，进度，环节，省内传输网络开通，审批未通过，加急推进</v>
+        <v>催,进度,环节,省内传输网络开通,审批未通过,加急推进</v>
       </c>
     </row>
     <row r="55">
@@ -2366,7 +2143,7 @@
         <v>建群、值班专家、客户经理加急</v>
       </c>
       <c r="H55" t="str">
-        <v>建群，拉群，值班专家，客户经理，加急，协助处理，烦请</v>
+        <v>建群,拉群,值班专家,客户经理,加急,协助处理,烦请</v>
       </c>
     </row>
     <row r="56">
@@ -2392,7 +2169,7 @@
         <v>包月/按量、账单、退订计费规则</v>
       </c>
       <c r="H56" t="str">
-        <v>资费，计费，账单，包月，扣费，多少钱，计费咨询，如何计费</v>
+        <v>资费,计费,账单,包月,扣费,多少钱,计费咨询,如何计费</v>
       </c>
     </row>
     <row r="57">
@@ -2418,7 +2195,7 @@
         <v>L4/L7、旗舰型、可用区、是否支持某特性</v>
       </c>
       <c r="H57" t="str">
-        <v>咨询，是否支持，规格，旗舰型，七层，四层，应用型，网络型，V4，V6，可用区</v>
+        <v>咨询,是否支持,规格,旗舰型,七层,四层,应用型,网络型,V4,V6,可用区</v>
       </c>
     </row>
     <row r="58">
@@ -2444,7 +2221,7 @@
         <v>转发是否实时生效、多可用区部署等</v>
       </c>
       <c r="H58" t="str">
-        <v>方案，架构，怎么配，转发策略修改，实时生效，业务方案</v>
+        <v>方案,架构,怎么配,转发策略修改,实时生效,业务方案</v>
       </c>
     </row>
     <row r="59">
@@ -2470,7 +2247,7 @@
         <v>控制台/API 创建 SLB 实例</v>
       </c>
       <c r="H59" t="str">
-        <v>开通，创建，订购，申购，创建实例，无法创建，API，接口文档</v>
+        <v>开通,创建,订购,申购,创建实例,无法创建,API,接口文档</v>
       </c>
     </row>
     <row r="60">
@@ -2496,7 +2273,7 @@
         <v>实例数、服务器组数量、访问控制组配额提升</v>
       </c>
       <c r="H60" t="str">
-        <v>配额，配额不足，提升配额，上限，提高到50，提高到70，服务器组数量</v>
+        <v>配额,配额不足,提升配额,上限,提高到50,提高到70,服务器组数量</v>
       </c>
     </row>
     <row r="61">
@@ -2522,7 +2299,7 @@
         <v>规格上架、安装交付、合规扫描</v>
       </c>
       <c r="H61" t="str">
-        <v>上架，安装交付，交付，旗舰型上架，端口关闭仍能扫到，华南广州</v>
+        <v>上架,安装交付,交付,旗舰型上架,端口关闭仍能扫到,华南广州</v>
       </c>
     </row>
     <row r="62">
@@ -2548,7 +2325,7 @@
         <v>退订待审核、开通失败、MOP 订单</v>
       </c>
       <c r="H62" t="str">
-        <v>退订，等待审核，MOP-T，订单编号，开通失败，订单状态</v>
+        <v>退订,等待审核,MOP-T,订单编号,开通失败,订单状态</v>
       </c>
     </row>
     <row r="63">
@@ -2574,7 +2351,7 @@
         <v>创建/修改监听、端口、协议</v>
       </c>
       <c r="H63" t="str">
-        <v>监听，创建监听，监听失败，端口，80，443，HTTP，HTTPS，TCP，UDP</v>
+        <v>监听,创建监听,监听失败,端口,80,443,HTTP,HTTPS,TCP,UDP</v>
       </c>
     </row>
     <row r="64">
@@ -2600,7 +2377,7 @@
         <v>添加后端、服务器组、权重</v>
       </c>
       <c r="H64" t="str">
-        <v>后端，服务器组，后端服务器组，添加后端，不能添加，绑定，权重，member</v>
+        <v>后端,服务器组,后端服务器组,添加后端,不能添加,绑定,权重,member</v>
       </c>
     </row>
     <row r="65">
@@ -2626,7 +2403,7 @@
         <v>探测失败、异常后端摘除</v>
       </c>
       <c r="H65" t="str">
-        <v>健康检查，探测，health，异常后端，检查间隔</v>
+        <v>健康检查,探测,health,异常后端,检查间隔</v>
       </c>
     </row>
     <row r="66">
@@ -2652,7 +2429,7 @@
         <v>URL/域名转发、规则优先级</v>
       </c>
       <c r="H66" t="str">
-        <v>转发，转发策略，规则，路由，域名转发，URL，优先级，修改转发</v>
+        <v>转发,转发策略,规则,路由,域名转发,URL,优先级,修改转发</v>
       </c>
     </row>
     <row r="67">
@@ -2678,7 +2455,7 @@
         <v>粘性、Cookie、轮询/加权/最小连接</v>
       </c>
       <c r="H67" t="str">
-        <v>会话保持，粘性，cookie，轮询，加权，最小连接，负载算法</v>
+        <v>会话保持,粘性,cookie,轮询,加权,最小连接,负载算法</v>
       </c>
     </row>
     <row r="68">
@@ -2704,7 +2481,7 @@
         <v>证书上传、SSL、TLS 卸载</v>
       </c>
       <c r="H68" t="str">
-        <v>证书，SSL，HTTPS，TLS，证书绑定，双向认证</v>
+        <v>证书,SSL,HTTPS,TLS,证书绑定,双向认证</v>
       </c>
     </row>
     <row r="69">
@@ -2730,7 +2507,7 @@
         <v>绑定 EIP、浮动 IP、内网 LB</v>
       </c>
       <c r="H69" t="str">
-        <v>VIP，公网，内网，EIP，浮动IP，公网IP，访问地址</v>
+        <v>VIP,公网,内网,EIP,浮动IP,公网IP,访问地址</v>
       </c>
     </row>
     <row r="70">
@@ -2756,7 +2533,7 @@
         <v>访问控制组、IP 白名单</v>
       </c>
       <c r="H70" t="str">
-        <v>访问控制，访问控制组，白名单，ACL，IP白名单</v>
+        <v>访问控制,访问控制组,白名单,ACL,IP白名单</v>
       </c>
     </row>
     <row r="71">
@@ -2782,7 +2559,7 @@
         <v>502/503/504、连接失败</v>
       </c>
       <c r="H71" t="str">
-        <v>不通，无法访问，502，503，504，连接失败，访问不了，访问异常</v>
+        <v>不通,无法访问,502,503,504,连接失败,访问不了,访问异常</v>
       </c>
     </row>
     <row r="72">
@@ -2808,7 +2585,7 @@
         <v>延迟高、超时</v>
       </c>
       <c r="H72" t="str">
-        <v>慢，超时，延迟，响应慢，卡顿</v>
+        <v>慢,超时,延迟,响应慢,卡顿</v>
       </c>
     </row>
     <row r="73">
@@ -2834,7 +2611,7 @@
         <v>大面积不可用、紧急验证</v>
       </c>
       <c r="H73" t="str">
-        <v>中断，不可用，业务影响，紧急，非常紧急</v>
+        <v>中断,不可用,业务影响,紧急,非常紧急</v>
       </c>
     </row>
     <row r="74">
@@ -2860,7 +2637,7 @@
         <v>后台核实、抓包定位</v>
       </c>
       <c r="H74" t="str">
-        <v>协查，排查，根因，抓包，协助核实，定位</v>
+        <v>协查,排查,根因,抓包,协助核实,定位</v>
       </c>
     </row>
     <row r="75">
@@ -2886,7 +2663,7 @@
         <v>包月退订、审核中订单</v>
       </c>
       <c r="H75" t="str">
-        <v>退订，取消，撤销，包月，等待审核</v>
+        <v>退订,取消,撤销,包月,等待审核</v>
       </c>
     </row>
     <row r="76">
@@ -2912,7 +2689,7 @@
         <v>删除 SLB、释放资源</v>
       </c>
       <c r="H76" t="str">
-        <v>删除，释放，销毁，下线</v>
+        <v>删除,释放,销毁,下线</v>
       </c>
     </row>
     <row r="77">
@@ -2938,7 +2715,7 @@
         <v>催交付、审批节点</v>
       </c>
       <c r="H77" t="str">
-        <v>催，进度，环节，加急，审批</v>
+        <v>催,进度,环节,加急,审批</v>
       </c>
     </row>
     <row r="78">
@@ -2964,243 +2741,2190 @@
         <v>OpenAPI/SDK 调用异常</v>
       </c>
       <c r="H78" t="str">
-        <v>API，接口，SDK，OpenAPI，调用失败，返回内容</v>
+        <v>API,接口,SDK,OpenAPI,调用失败,返回内容</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B79" t="str">
+        <v>discover</v>
+      </c>
+      <c r="C79" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="D79" t="str">
+        <v>了解 VPC 能力、网段规划、多 VPC/混合云组网；资费与配额咨询（报障类请结合请求场景=报障与恢复）</v>
+      </c>
+      <c r="E79" t="str">
+        <v>discover-intro</v>
+      </c>
+      <c r="F79" t="str">
+        <v>产品与能力咨询</v>
+      </c>
+      <c r="G79" t="str">
+        <v>VPC 功能咨询、是否支持、子网回收通知、功能使用说明</v>
+      </c>
+      <c r="H79" t="str">
+        <v>咨询,了解,VPC,虚拟私有云,专有网络,是否支持,产品介绍,IPv6,能力,VPC功能使用咨询,功能使用咨询,子网回收,回收子网,短信提示</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B80" t="str">
+        <v>discover</v>
+      </c>
+      <c r="C80" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="D80" t="str">
+        <v>了解 VPC 能力、网段规划、多 VPC/混合云组网；资费与配额咨询（报障类请结合请求场景=报障与恢复）</v>
+      </c>
+      <c r="E80" t="str">
+        <v>discover-rules</v>
+      </c>
+      <c r="F80" t="str">
+        <v>业务规则与全局咨询</v>
+      </c>
+      <c r="G80" t="str">
+        <v>业务规则咨询、全局流转、VPC 日志/规格规则、政务网互通规则</v>
+      </c>
+      <c r="H80" t="str">
+        <v>业务规则咨询,全局流转,VPC业务规则咨询,虚拟私有云业务规则咨询,业务规则,VPC日志,vpC日志,规则咨询,查询</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B81" t="str">
+        <v>discover</v>
+      </c>
+      <c r="C81" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="D81" t="str">
+        <v>了解 VPC 能力、网段规划、多 VPC/混合云组网；资费与配额咨询（报障类请结合请求场景=报障与恢复）</v>
+      </c>
+      <c r="E81" t="str">
+        <v>discover-cidr</v>
+      </c>
+      <c r="F81" t="str">
+        <v>网段与容量规划</v>
+      </c>
+      <c r="G81" t="str">
+        <v>CIDR、掩码、子网数量、网段重叠、特殊网段申请</v>
+      </c>
+      <c r="H81" t="str">
+        <v>网段,CIDR,规划,掩码,重叠,网段冲突,子网数量,容量,地址段,网段复用,7.0.0.0,192.168,10.</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B82" t="str">
+        <v>discover</v>
+      </c>
+      <c r="C82" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="D82" t="str">
+        <v>了解 VPC 能力、网段规划、多 VPC/混合云组网；资费与配额咨询（报障类请结合请求场景=报障与恢复）</v>
+      </c>
+      <c r="E82" t="str">
+        <v>discover-architecture</v>
+      </c>
+      <c r="F82" t="str">
+        <v>组网与架构咨询</v>
+      </c>
+      <c r="G82" t="str">
+        <v>多 VPC、多地域、与 IDC/专线/VPN/政务网组网拓扑</v>
+      </c>
+      <c r="H82" t="str">
+        <v>组网,架构,方案,混合云,三层,拓扑,多VPC,跨地域,政务网,打通互访</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B83" t="str">
+        <v>provision</v>
+      </c>
+      <c r="C83" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="D83" t="str">
+        <v>创建 VPC/子网、安装交付、可用区选择、配额权限、网段变更</v>
+      </c>
+      <c r="E83" t="str">
+        <v>provision-create</v>
+      </c>
+      <c r="F83" t="str">
+        <v>创建VPC与子网</v>
+      </c>
+      <c r="G83" t="str">
+        <v>新建 VPC、子网、VPC 订购开通</v>
+      </c>
+      <c r="H83" t="str">
+        <v>创建,新建,开通,创建VPC,创建子网,创建失败,无法创建,VPC订购,VPC订购/开通,订购/开通</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B84" t="str">
+        <v>provision</v>
+      </c>
+      <c r="C84" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="D84" t="str">
+        <v>创建 VPC/子网、安装交付、可用区选择、配额权限、网段变更</v>
+      </c>
+      <c r="E84" t="str">
+        <v>provision-delivery</v>
+      </c>
+      <c r="F84" t="str">
+        <v>安装交付与权限开通</v>
+      </c>
+      <c r="G84" t="str">
+        <v>VPC 安装交付、资源池订购权限、后台协助开通</v>
+      </c>
+      <c r="H84" t="str">
+        <v>VPC安装交付,安装交付,虚拟私有云安装交付,开通权限,订购权限,开通对应资源池,后台协助开通,资源池的订购权限</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B85" t="str">
+        <v>provision</v>
+      </c>
+      <c r="C85" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="D85" t="str">
+        <v>创建 VPC/子网、安装交付、可用区选择、配额权限、网段变更</v>
+      </c>
+      <c r="E85" t="str">
+        <v>provision-az-subnet</v>
+      </c>
+      <c r="F85" t="str">
+        <v>可用区与子网选择</v>
+      </c>
+      <c r="G85" t="str">
+        <v>子网灰掉、VPC 子网无法选择、AZ/资源池限制</v>
+      </c>
+      <c r="H85" t="str">
+        <v>可用区,AZ,子网无法选择,VPC子网无法选择,选不了,灰掉,资源池,华东,苏州,华中,长沙</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B86" t="str">
+        <v>provision</v>
+      </c>
+      <c r="C86" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="D86" t="str">
+        <v>创建 VPC/子网、安装交付、可用区选择、配额权限、网段变更</v>
+      </c>
+      <c r="E86" t="str">
+        <v>provision-quota</v>
+      </c>
+      <c r="F86" t="str">
+        <v>配额与权限</v>
+      </c>
+      <c r="G86" t="str">
+        <v>VPC/子网/对等连接配额提升、灰度与权限申请（含误挂「退订」节点的配额单）</v>
+      </c>
+      <c r="H86" t="str">
+        <v>配额,配额不足,配额提升,提高配额,配额至,提升到,权限,权限不足,RAM,IAM,订单失败,上限,满上限,灰度申请,申请提升vpc配额,VPC配额</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B87" t="str">
+        <v>provision</v>
+      </c>
+      <c r="C87" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="D87" t="str">
+        <v>创建 VPC/子网、安装交付、可用区选择、配额权限、网段变更</v>
+      </c>
+      <c r="E87" t="str">
+        <v>provision-subnet-change</v>
+      </c>
+      <c r="F87" t="str">
+        <v>变更网段与VPC业务变更</v>
+      </c>
+      <c r="G87" t="str">
+        <v>VPC 业务变更、删除修改、子网不互通、添加/修改子网</v>
+      </c>
+      <c r="H87" t="str">
+        <v>添加子网,网段变更,VPC变更,VPC业务变更,虚拟私有云业务变更,扩容,修改网段,子网扩容,变更子网,VPC删除修改,删除修改操作,子网不互通,两台主机,不互通</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B88" t="str">
+        <v>route-nat</v>
+      </c>
+      <c r="C88" t="str">
+        <v>路由与网关</v>
+      </c>
+      <c r="D88" t="str">
+        <v>路由表、NAT 网关、对等连接、终端节点</v>
+      </c>
+      <c r="E88" t="str">
+        <v>route-table</v>
+      </c>
+      <c r="F88" t="str">
+        <v>路由表与默认路由</v>
+      </c>
+      <c r="G88" t="str">
+        <v>路由不通、缺默认路由、路由优先级、自定义路由</v>
+      </c>
+      <c r="H88" t="str">
+        <v>路由表,默认路由,路由策略,路由规则,下一跳,路由不通</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B89" t="str">
+        <v>route-nat</v>
+      </c>
+      <c r="C89" t="str">
+        <v>路由与网关</v>
+      </c>
+      <c r="D89" t="str">
+        <v>路由表、NAT 网关、对等连接、终端节点</v>
+      </c>
+      <c r="E89" t="str">
+        <v>route-nat</v>
+      </c>
+      <c r="F89" t="str">
+        <v>NAT网关</v>
+      </c>
+      <c r="G89" t="str">
+        <v>SNAT/DNAT、NAT 创建绑定、出网路径</v>
+      </c>
+      <c r="H89" t="str">
+        <v>NAT,NAT网关,SNAT,DNAT,NAT创建,绑定NAT</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B90" t="str">
+        <v>route-nat</v>
+      </c>
+      <c r="C90" t="str">
+        <v>路由与网关</v>
+      </c>
+      <c r="D90" t="str">
+        <v>路由表、NAT 网关、对等连接、终端节点</v>
+      </c>
+      <c r="E90" t="str">
+        <v>route-peering</v>
+      </c>
+      <c r="F90" t="str">
+        <v>对等连接与云互联</v>
+      </c>
+      <c r="G90" t="str">
+        <v>跨 VPC、跨账号 Peering、对等连接配额/满额</v>
+      </c>
+      <c r="H90" t="str">
+        <v>对等连接,Peering,云互联,跨VPC,跨账号,跨账户,互联,对等连接满,对等连接上限,满上限</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B91" t="str">
+        <v>route-nat</v>
+      </c>
+      <c r="C91" t="str">
+        <v>路由与网关</v>
+      </c>
+      <c r="D91" t="str">
+        <v>路由表、NAT 网关、对等连接、终端节点</v>
+      </c>
+      <c r="E91" t="str">
+        <v>route-endpoint</v>
+      </c>
+      <c r="F91" t="str">
+        <v>终端节点与私有连接</v>
+      </c>
+      <c r="G91" t="str">
+        <v>PrivateLink、终端节点、私有服务访问</v>
+      </c>
+      <c r="H91" t="str">
+        <v>终端节点,PrivateLink,私有连接,终端节点服务,VPC终端</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B92" t="str">
+        <v>security</v>
+      </c>
+      <c r="C92" t="str">
+        <v>安全与访问控制</v>
+      </c>
+      <c r="D92" t="str">
+        <v>安全组、网络 ACL、VPC 语境下的访问策略</v>
+      </c>
+      <c r="E92" t="str">
+        <v>security-group</v>
+      </c>
+      <c r="F92" t="str">
+        <v>安全组配置与异常</v>
+      </c>
+      <c r="G92" t="str">
+        <v>安全组不生效、放通仍不通、与 ECS 网卡/虚拟网卡联动</v>
+      </c>
+      <c r="H92" t="str">
+        <v>安全组,安全组配置异常,不生效,放通,端口,入方向,出方向,网卡,虚拟网卡,updatePortSecurityGroups,修改虚拟网卡安全组</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B93" t="str">
+        <v>security</v>
+      </c>
+      <c r="C93" t="str">
+        <v>安全与访问控制</v>
+      </c>
+      <c r="D93" t="str">
+        <v>安全组、网络 ACL、VPC 语境下的访问策略</v>
+      </c>
+      <c r="E93" t="str">
+        <v>security-acl</v>
+      </c>
+      <c r="F93" t="str">
+        <v>网络ACL</v>
+      </c>
+      <c r="G93" t="str">
+        <v>子网 ACL 满额、规则顺序、ACL 拦截</v>
+      </c>
+      <c r="H93" t="str">
+        <v>网络ACL,ACL,子网ACL,访问控制列表,规则顺序,ACL规则,ACL规则已满,acl规则已满,规则已满</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B94" t="str">
+        <v>security</v>
+      </c>
+      <c r="C94" t="str">
+        <v>安全与访问控制</v>
+      </c>
+      <c r="D94" t="str">
+        <v>安全组、网络 ACL、VPC 语境下的访问策略</v>
+      </c>
+      <c r="E94" t="str">
+        <v>security-policy</v>
+      </c>
+      <c r="F94" t="str">
+        <v>封堵与白名单</v>
+      </c>
+      <c r="G94" t="str">
+        <v>平台封堵、出口策略、内网白名单</v>
+      </c>
+      <c r="H94" t="str">
+        <v>封堵,白名单,黑名单,出口策略,内网访问</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B95" t="str">
+        <v>operate</v>
+      </c>
+      <c r="C95" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="D95" t="str">
+        <v>内网/出网不通、云主机换 VPC、HAVIP、链路质量</v>
+      </c>
+      <c r="E95" t="str">
+        <v>operate-internal</v>
+      </c>
+      <c r="F95" t="str">
+        <v>内网互通异常</v>
+      </c>
+      <c r="G95" t="str">
+        <v>同 VPC 跨子网、跨 AZ、EOS/内网地址不通</v>
+      </c>
+      <c r="H95" t="str">
+        <v>内网不通,子网不通,跨子网,跨AZ,ping不通,内网访问,互通,内网地址不通,eos内网,endpoint地址</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B96" t="str">
+        <v>operate</v>
+      </c>
+      <c r="C96" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="D96" t="str">
+        <v>内网/出网不通、云主机换 VPC、HAVIP、链路质量</v>
+      </c>
+      <c r="E96" t="str">
+        <v>operate-egress</v>
+      </c>
+      <c r="F96" t="str">
+        <v>出网与入网异常</v>
+      </c>
+      <c r="G96" t="str">
+        <v>经 NAT/EIP 仍不通、外网访问异常</v>
+      </c>
+      <c r="H96" t="str">
+        <v>出网,入网,无法上网,外网不通,访问外网,无法连接外网,linux系统主机无法连接外网</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B97" t="str">
+        <v>operate</v>
+      </c>
+      <c r="C97" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="D97" t="str">
+        <v>内网/出网不通、云主机换 VPC、HAVIP、链路质量</v>
+      </c>
+      <c r="E97" t="str">
+        <v>operate-ecs</v>
+      </c>
+      <c r="F97" t="str">
+        <v>与云主机网卡联动</v>
+      </c>
+      <c r="G97" t="str">
+        <v>更换 VPC、多网卡路由、云主机迁移 VPC</v>
+      </c>
+      <c r="H97" t="str">
+        <v>更换VPC,云主机更换VPC,多网卡,主网卡,弹性网卡,ENI,网卡绑定,云主机,ECS,部署的网站</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B98" t="str">
+        <v>operate</v>
+      </c>
+      <c r="C98" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="D98" t="str">
+        <v>内网/出网不通、云主机换 VPC、HAVIP、链路质量</v>
+      </c>
+      <c r="E98" t="str">
+        <v>operate-havip</v>
+      </c>
+      <c r="F98" t="str">
+        <v>HAVIP与高可用</v>
+      </c>
+      <c r="G98" t="str">
+        <v>VPC 下 HAVIP 无法使用、HA VIP 异常</v>
+      </c>
+      <c r="H98" t="str">
+        <v>HAVIP,HA VIP,HAVIP无法使用,havip,高可用IP</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B99" t="str">
+        <v>operate</v>
+      </c>
+      <c r="C99" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="D99" t="str">
+        <v>内网/出网不通、云主机换 VPC、HAVIP、链路质量</v>
+      </c>
+      <c r="E99" t="str">
+        <v>operate-quality</v>
+      </c>
+      <c r="F99" t="str">
+        <v>时延与链路质量</v>
+      </c>
+      <c r="G99" t="str">
+        <v>丢包、延迟、抖动、不稳定</v>
+      </c>
+      <c r="H99" t="str">
+        <v>丢包,延迟,抖动,慢,不稳定,质量差,卡顿</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B100" t="str">
+        <v>hybrid</v>
+      </c>
+      <c r="C100" t="str">
+        <v>混合云与专线接入</v>
+      </c>
+      <c r="D100" t="str">
+        <v>专线接入 VPC、跨账号/跨资源池；专线开通交付归云专线产品</v>
+      </c>
+      <c r="E100" t="str">
+        <v>hybrid-dc</v>
+      </c>
+      <c r="F100" t="str">
+        <v>专线接入VPC</v>
+      </c>
+      <c r="G100" t="str">
+        <v>用户侧子网、边界网关、互联地址（VPC 配置侧）</v>
+      </c>
+      <c r="H100" t="str">
+        <v>专线接入,云专线,用户侧子网,边界网关,互联地址,dummy</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B101" t="str">
+        <v>hybrid</v>
+      </c>
+      <c r="C101" t="str">
+        <v>混合云与专线接入</v>
+      </c>
+      <c r="D101" t="str">
+        <v>专线接入 VPC、跨账号/跨资源池；专线开通交付归云专线产品</v>
+      </c>
+      <c r="E101" t="str">
+        <v>hybrid-cross-account</v>
+      </c>
+      <c r="F101" t="str">
+        <v>跨账号与跨资源池</v>
+      </c>
+      <c r="G101" t="str">
+        <v>跨资源池路由、同一 VPC、跨账户对接</v>
+      </c>
+      <c r="H101" t="str">
+        <v>跨资源池,同一vpc,跨账号,跨账户,用户子网相同,同一云账号</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B102" t="str">
+        <v>hybrid</v>
+      </c>
+      <c r="C102" t="str">
+        <v>混合云与专线接入</v>
+      </c>
+      <c r="D102" t="str">
+        <v>专线接入 VPC、跨账号/跨资源池；专线开通交付归云专线产品</v>
+      </c>
+      <c r="E102" t="str">
+        <v>hybrid-vpn</v>
+      </c>
+      <c r="F102" t="str">
+        <v>VPN与其他接入</v>
+      </c>
+      <c r="G102" t="str">
+        <v>VPN 网关、IPsec、SSL VPN 接入 VPC</v>
+      </c>
+      <c r="H102" t="str">
+        <v>VPN,IPsec,SSL VPN,VPN网关,隧道</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B103" t="str">
+        <v>lifecycle</v>
+      </c>
+      <c r="C103" t="str">
+        <v>变更退订与治理</v>
+      </c>
+      <c r="D103" t="str">
+        <v>迁移割接、退订释放、账单计费</v>
+      </c>
+      <c r="E103" t="str">
+        <v>lifecycle-change</v>
+      </c>
+      <c r="F103" t="str">
+        <v>变更与迁移</v>
+      </c>
+      <c r="G103" t="str">
+        <v>VPC 迁移、割接（非业务变更类见 provision-subnet-change）</v>
+      </c>
+      <c r="H103" t="str">
+        <v>迁移,割接,搬迁,切换</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B104" t="str">
+        <v>lifecycle</v>
+      </c>
+      <c r="C104" t="str">
+        <v>变更退订与治理</v>
+      </c>
+      <c r="D104" t="str">
+        <v>迁移割接、退订释放、账单计费</v>
+      </c>
+      <c r="E104" t="str">
+        <v>lifecycle-release</v>
+      </c>
+      <c r="F104" t="str">
+        <v>退订与释放</v>
+      </c>
+      <c r="G104" t="str">
+        <v>删除 VPC、资源退订释放、依赖残留（纯配额类见 provision-quota）</v>
+      </c>
+      <c r="H104" t="str">
+        <v>VPC退订,退订VPC,释放VPC,删除VPC,无法删除,销毁,依赖,残留,已经全部退订</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B105" t="str">
+        <v>lifecycle</v>
+      </c>
+      <c r="C105" t="str">
+        <v>变更退订与治理</v>
+      </c>
+      <c r="D105" t="str">
+        <v>迁移割接、退订释放、账单计费</v>
+      </c>
+      <c r="E105" t="str">
+        <v>lifecycle-billing</v>
+      </c>
+      <c r="F105" t="str">
+        <v>账单与计费咨询</v>
+      </c>
+      <c r="G105" t="str">
+        <v>VPC 相关计费项、账单、扣费规则</v>
+      </c>
+      <c r="H105" t="str">
+        <v>账单,计费,扣费,资费,出账,费用,计费咨询</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H105"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C13"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>问题类型名称</v>
+      </c>
+      <c r="B1" t="str">
+        <v>问题类型说明</v>
+      </c>
+      <c r="C1" t="str">
+        <v>参考关键词</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>可用性/连通性故障</v>
+      </c>
+      <c r="B2" t="str">
+        <v>业务完全中断、网络不通、服务崩溃、IP 封堵、黑洞；云主机无法启动、专线完全不通、IP 被封等</v>
+      </c>
+      <c r="C2" t="str">
+        <v>不通,中断,崩溃,不可用,完全打不开,服务挂了,ping不通,PING不通,连接失败,时通时断,封堵,黑洞,底层异常,异网故障</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>性能问题</v>
+      </c>
+      <c r="B3" t="str">
+        <v>服务可用但响应慢、卡顿、延迟高、丢包、重传；API 响应慢、页面卡顿、视频卡顿等</v>
+      </c>
+      <c r="C3" t="str">
+        <v>慢,卡顿,延迟,超时,响应慢,加载慢,丢包,重传,抖动</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>计费与账单</v>
+      </c>
+      <c r="B4" t="str">
+        <v>费用异常、扣费错误、账单金额不对等计费问题（单纯账单查询、计费规则咨询不归此类）</v>
+      </c>
+      <c r="C4" t="str">
+        <v>多扣,少扣,金额不对,账单错误,扣费异常,欠费误判,费用多收了,计费错误</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>配额与权限申请</v>
+      </c>
+      <c r="B5" t="str">
+        <v>主动申请提升配额、权限、解售罄、轻载 IP、灰度、解除 8:1 限制、带宽扩容等</v>
+      </c>
+      <c r="C5" t="str">
+        <v>配额申请,提升配额,IP配额,带宽配额,解售罄,上架,轻载IP,轻载通道,灰度权限,解除8:1限制,取消8:1,开通灰度,大带宽权限,申请IP,扩容带宽,带宽提升,增加IP数量</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>资源开通与创建</v>
+      </c>
+      <c r="B6" t="str">
+        <v>创建/开通资源时技术失败（非配额问题）；创建实例失败、开通 CDN 超时、订购报错等</v>
+      </c>
+      <c r="C6" t="str">
+        <v>创建失败,开通失败,申购失败,实例启动失败,无法创建,订购失败</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>配置与操作</v>
+      </c>
+      <c r="B7" t="str">
+        <v>已有资源的绑定、解绑、修改配置等操作失败或异常（正常操作咨询不归此类）</v>
+      </c>
+      <c r="C7" t="str">
+        <v>绑定失败,解绑失败,修改配置失败,调整带宽失败,关联失败,变更失败,配置报错,操作报错</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>退订与释放</v>
+      </c>
+      <c r="B8" t="str">
+        <v>资源退订、释放、删除操作失败或异常，或明确要求执行退订（正常退订咨询不归此类）</v>
+      </c>
+      <c r="C8" t="str">
+        <v>无法退订,退订失败,释放失败,删除失败,退订报错,删不掉,销毁失败,请帮我退订,请帮忙释放</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>界面与操作易用性</v>
+      </c>
+      <c r="B9" t="str">
+        <v>控制台界面、交互、提示等体验问题（不涉及功能缺失）；按钮难找、提示不清、操作步骤繁琐等</v>
+      </c>
+      <c r="C9" t="str">
+        <v>控制台,体验差,操作繁琐,按钮难找,提示不清,界面乱,不方便</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>产品功能需求</v>
+      </c>
+      <c r="B10" t="str">
+        <v>提出新功能或现有功能增强的建议；希望增加批量删除、建议支持 IPv6 等</v>
+      </c>
+      <c r="C10" t="str">
+        <v>希望,建议,能不能,需要支持,增加功能</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>产品功能咨询</v>
+      </c>
+      <c r="B11" t="str">
+        <v>询问现有功能用法、规则、信息、进度、账单查询、计费规则、如何退订等</v>
+      </c>
+      <c r="C11" t="str">
+        <v>咨询,请问,如何,怎么,怎样,是否支持,规则,指导,查询,核实,进度,掩码,配置值,帮助文档,操作步骤,退订流程,对端拒绝,对端服务器,被对方重置</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>人工服务与流程</v>
+      </c>
+      <c r="B12" t="str">
+        <v>客服响应、工单流转、服务态度、催办等问题；要求出具故障报告等</v>
+      </c>
+      <c r="C12" t="str">
+        <v>客服,工单,等待,态度差,流程长,没人回,赔偿,催办,故障报告</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>其他</v>
+      </c>
+      <c r="B13" t="str">
+        <v>无法归类的技术问题或无技术问题的纯情绪反馈；纯情绪抱怨、无关内容</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D40"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>产品Key</v>
+      </c>
+      <c r="B1" t="str">
+        <v>请求节点服务类型</v>
+      </c>
+      <c r="C1" t="str">
+        <v>一级ID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>一级名称</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>eip</v>
+      </c>
+      <c r="B2" t="str">
+        <v>产品咨询</v>
+      </c>
+      <c r="C2" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D2" t="str">
+        <v>认知与选型</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>eip</v>
+      </c>
+      <c r="B3" t="str">
+        <v>产品使用问题</v>
+      </c>
+      <c r="C3" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D3" t="str">
+        <v>业务使用与连通</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>eip</v>
+      </c>
+      <c r="B4" t="str">
+        <v>产品功能</v>
+      </c>
+      <c r="C4" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D4" t="str">
+        <v>认知与选型</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>eip</v>
+      </c>
+      <c r="B5" t="str">
+        <v>产品使用</v>
+      </c>
+      <c r="C5" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D5" t="str">
+        <v>业务使用与连通</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>eip</v>
+      </c>
+      <c r="B6" t="str">
+        <v>其他</v>
+      </c>
+      <c r="C6" t="str">
+        <v>service</v>
+      </c>
+      <c r="D6" t="str">
+        <v>服务与体验</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B7" t="str">
+        <v>产品咨询</v>
+      </c>
+      <c r="C7" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D7" t="str">
+        <v>方案与商务</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B8" t="str">
+        <v>产品使用问题</v>
+      </c>
+      <c r="C8" t="str">
+        <v>access</v>
+      </c>
+      <c r="D8" t="str">
+        <v>接入与配置</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B9" t="str">
+        <v>产品功能</v>
+      </c>
+      <c r="C9" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D9" t="str">
+        <v>方案与商务</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B10" t="str">
+        <v>产品使用</v>
+      </c>
+      <c r="C10" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D10" t="str">
+        <v>运行与质量</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B11" t="str">
+        <v>业务方案支撑</v>
+      </c>
+      <c r="C11" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D11" t="str">
+        <v>方案与商务</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B12" t="str">
+        <v>开通与权限申请</v>
+      </c>
+      <c r="C12" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D12" t="str">
+        <v>开通与交付</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B13" t="str">
+        <v>报障排障</v>
+      </c>
+      <c r="C13" t="str">
+        <v>incident</v>
+      </c>
+      <c r="D13" t="str">
+        <v>故障与应急</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B14" t="str">
+        <v>计费与账务</v>
+      </c>
+      <c r="C14" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D14" t="str">
+        <v>方案与商务</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B15" t="str">
+        <v>协查与跟进</v>
+      </c>
+      <c r="C15" t="str">
+        <v>service</v>
+      </c>
+      <c r="D15" t="str">
+        <v>服务与流程</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>dc</v>
+      </c>
+      <c r="B16" t="str">
+        <v>其他</v>
+      </c>
+      <c r="C16" t="str">
+        <v>service</v>
+      </c>
+      <c r="D16" t="str">
+        <v>服务与流程</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B17" t="str">
+        <v>产品咨询</v>
+      </c>
+      <c r="C17" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D17" t="str">
+        <v>认知与方案</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B18" t="str">
+        <v>产品功能</v>
+      </c>
+      <c r="C18" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D18" t="str">
+        <v>认知与方案</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B19" t="str">
+        <v>产品使用问题</v>
+      </c>
+      <c r="C19" t="str">
+        <v>configure</v>
+      </c>
+      <c r="D19" t="str">
+        <v>监听与转发配置</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B20" t="str">
+        <v>产品使用</v>
+      </c>
+      <c r="C20" t="str">
+        <v>configure</v>
+      </c>
+      <c r="D20" t="str">
+        <v>监听与转发配置</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B21" t="str">
+        <v>业务方案支撑</v>
+      </c>
+      <c r="C21" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D21" t="str">
+        <v>认知与方案</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B22" t="str">
+        <v>开通与权限申请</v>
+      </c>
+      <c r="C22" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D22" t="str">
+        <v>开通与上架</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B23" t="str">
+        <v>报障排障</v>
+      </c>
+      <c r="C23" t="str">
+        <v>incident</v>
+      </c>
+      <c r="D23" t="str">
+        <v>故障与应急</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B24" t="str">
+        <v>计费与账务</v>
+      </c>
+      <c r="C24" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D24" t="str">
+        <v>认知与方案</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B25" t="str">
+        <v>协查与跟进</v>
+      </c>
+      <c r="C25" t="str">
+        <v>service</v>
+      </c>
+      <c r="D25" t="str">
+        <v>服务与流程</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B26" t="str">
+        <v>其他</v>
+      </c>
+      <c r="C26" t="str">
+        <v>service</v>
+      </c>
+      <c r="D26" t="str">
+        <v>服务与流程</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B27" t="str">
+        <v>VPC</v>
+      </c>
+      <c r="C27" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D27" t="str">
+        <v>创建与基础资源</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B28" t="str">
+        <v>虚拟私有云</v>
+      </c>
+      <c r="C28" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D28" t="str">
+        <v>创建与基础资源</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B29" t="str">
+        <v>全局流转</v>
+      </c>
+      <c r="C29" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D29" t="str">
+        <v>认知与组网规划</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B30" t="str">
+        <v>云主机</v>
+      </c>
+      <c r="C30" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D30" t="str">
+        <v>业务连通与运行</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B31" t="str">
+        <v>产品咨询</v>
+      </c>
+      <c r="C31" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D31" t="str">
+        <v>认知与组网规划</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B32" t="str">
+        <v>产品功能</v>
+      </c>
+      <c r="C32" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D32" t="str">
+        <v>认知与组网规划</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B33" t="str">
+        <v>产品使用问题</v>
+      </c>
+      <c r="C33" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D33" t="str">
+        <v>业务连通与运行</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B34" t="str">
+        <v>产品使用</v>
+      </c>
+      <c r="C34" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D34" t="str">
+        <v>创建与基础资源</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B35" t="str">
+        <v>业务方案支撑</v>
+      </c>
+      <c r="C35" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D35" t="str">
+        <v>认知与组网规划</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B36" t="str">
+        <v>资源申请与开通</v>
+      </c>
+      <c r="C36" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D36" t="str">
+        <v>创建与基础资源</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B37" t="str">
+        <v>报障与恢复</v>
+      </c>
+      <c r="C37" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D37" t="str">
+        <v>业务连通与运行</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B38" t="str">
+        <v>费用与账务</v>
+      </c>
+      <c r="C38" t="str">
+        <v>lifecycle</v>
+      </c>
+      <c r="D38" t="str">
+        <v>变更退订与治理</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B39" t="str">
+        <v>进度查询与协同</v>
+      </c>
+      <c r="C39" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D39" t="str">
+        <v>创建与基础资源</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B40" t="str">
+        <v>其他</v>
+      </c>
+      <c r="C40" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D40" t="str">
+        <v>业务连通与运行</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D40"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:F37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>请求场景名称</v>
+        <v>产品Key</v>
       </c>
       <c r="B1" t="str">
-        <v>请求场景说明</v>
+        <v>请求节点问题子类</v>
       </c>
       <c r="C1" t="str">
-        <v>参考关键词</v>
+        <v>一级ID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>一级名称</v>
+      </c>
+      <c r="E1" t="str">
+        <v>二级ID</v>
+      </c>
+      <c r="F1" t="str">
+        <v>二级名称</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>报障与恢复</v>
+        <v>eip</v>
       </c>
       <c r="B2" t="str">
-        <v>用户认为现网已有异常（不可用、报错、中断、安全攻击影响业务等），核心诉求是排查并恢复，而非单纯问规则或进度</v>
+        <v>IP无法访问</v>
       </c>
       <c r="C2" t="str">
-        <v>故障，报障，不通，异常，中断，不可用，报错，502，503，宕机，封堵，攻击，无法访问</v>
+        <v>operate</v>
+      </c>
+      <c r="D2" t="str">
+        <v>业务使用与连通</v>
+      </c>
+      <c r="E2" t="str">
+        <v>operate-access</v>
+      </c>
+      <c r="F2" t="str">
+        <v>公网访问不通或不稳定、丢包</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>资源申请与开通</v>
+        <v>eip</v>
       </c>
       <c r="B3" t="str">
-        <v>用户主动发起资源或权限类申请：开通、配额、权限、灰度、上架/解售罄、解除限制、扩容申购等</v>
+        <v>产品功能</v>
       </c>
       <c r="C3" t="str">
-        <v>开通，申请，配额，权限，灰度，上架，解售罄，解除限制，申购，创建，扩容，授权</v>
+        <v>discover</v>
+      </c>
+      <c r="D3" t="str">
+        <v>认知与选型</v>
+      </c>
+      <c r="E3" t="str">
+        <v>discover-intro</v>
+      </c>
+      <c r="F3" t="str">
+        <v>产品与规格咨询</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>进度查询与协同</v>
+        <v>eip</v>
       </c>
       <c r="B4" t="str">
-        <v>用户跟进已有工单/订单/施工，或请云侧协助操作、协查、补材料；重点在进度与协同，而非首次报障或新开通</v>
+        <v>产品咨询</v>
       </c>
       <c r="C4" t="str">
-        <v>催办，进度，协查，跟进，环节，审批，协助处理，补充材料，建群，何时完成</v>
+        <v>discover</v>
+      </c>
+      <c r="D4" t="str">
+        <v>认知与选型</v>
+      </c>
+      <c r="E4" t="str">
+        <v>discover-intro</v>
+      </c>
+      <c r="F4" t="str">
+        <v>产品与规格咨询</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>业务方案支撑</v>
+        <v>eip</v>
       </c>
       <c r="B5" t="str">
-        <v>用户需要架构、选型、迁移/割接/落地等业务方案层面的支撑，超出单点产品 FAQ</v>
+        <v>其他</v>
       </c>
       <c r="C5" t="str">
-        <v>方案，架构，选型，落地，迁移，割接，业务咨询，组网，规划设计</v>
+        <v>operate</v>
+      </c>
+      <c r="D5" t="str">
+        <v>业务使用与连通</v>
+      </c>
+      <c r="E5" t="str">
+        <v>operate-quality</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>产品能力咨询</v>
+        <v>dc</v>
       </c>
       <c r="B6" t="str">
-        <v>用户了解产品能做什么、规格边界、是否支持、资费模型对比等认知与决策信息，不要求立刻开通或排障</v>
+        <v>产品咨询</v>
       </c>
       <c r="C6" t="str">
-        <v>咨询，是否支持，规格，能力，功能说明，产品介绍，对比，多少钱</v>
+        <v>discover</v>
+      </c>
+      <c r="D6" t="str">
+        <v>方案与商务</v>
+      </c>
+      <c r="E6" t="str">
+        <v>discover-capability</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>使用与配置指导</v>
+        <v>dc</v>
       </c>
       <c r="B7" t="str">
-        <v>用户需要操作步骤、配置方法、最佳实践指导；无报障、非大型方案设计</v>
+        <v>产品功能</v>
       </c>
       <c r="C7" t="str">
-        <v>怎么用，如何配置，操作步骤，配置方法，最佳实践，教程，指导</v>
+        <v>discover</v>
+      </c>
+      <c r="D7" t="str">
+        <v>方案与商务</v>
+      </c>
+      <c r="E7" t="str">
+        <v>discover-capability</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>费用与账务</v>
+        <v>dc</v>
       </c>
       <c r="B8" t="str">
-        <v>用户围绕账单、扣费、退费、发票、对账、资费核算提问或申诉，主诉在钱与账</v>
+        <v>IP无法访问</v>
       </c>
       <c r="C8" t="str">
-        <v>账单，计费，扣费，退费，发票，对账，欠费，资费，出账，冲销</v>
+        <v>operate</v>
+      </c>
+      <c r="D8" t="str">
+        <v>运行与质量</v>
+      </c>
+      <c r="E8" t="str">
+        <v>operate-connect</v>
+      </c>
+      <c r="F8" t="str">
+        <v>连通性异常</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>服务投诉与升级</v>
+        <v>dc</v>
       </c>
       <c r="B9" t="str">
-        <v>用户对客服态度、响应时效、处理流程不满，或要求投诉、升级、回访；主诉在服务交付过程，非产品故障</v>
+        <v>其他</v>
       </c>
       <c r="C9" t="str">
-        <v>投诉，不满，态度，服务差，升级，回访，督办，响应慢，无人跟进</v>
+        <v>operate</v>
+      </c>
+      <c r="D9" t="str">
+        <v>运行与质量</v>
+      </c>
+      <c r="E9" t="str">
+        <v>operate-connect</v>
+      </c>
+      <c r="F9" t="str">
+        <v>连通性异常</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B10" t="str">
+        <v>产品咨询</v>
+      </c>
+      <c r="C10" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D10" t="str">
+        <v>认知与方案</v>
+      </c>
+      <c r="E10" t="str">
+        <v>discover-capability</v>
+      </c>
+      <c r="F10" t="str">
+        <v>能力与规格咨询</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B11" t="str">
+        <v>产品功能</v>
+      </c>
+      <c r="C11" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D11" t="str">
+        <v>认知与方案</v>
+      </c>
+      <c r="E11" t="str">
+        <v>discover-capability</v>
+      </c>
+      <c r="F11" t="str">
+        <v>能力与规格咨询</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B12" t="str">
+        <v>IP无法访问</v>
+      </c>
+      <c r="C12" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D12" t="str">
+        <v>业务访问与质量</v>
+      </c>
+      <c r="E12" t="str">
+        <v>operate-unavailable</v>
+      </c>
+      <c r="F12" t="str">
+        <v>访问不通与错误码</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>slb</v>
+      </c>
+      <c r="B13" t="str">
+        <v>其他</v>
+      </c>
+      <c r="C13" t="str">
+        <v>configure</v>
+      </c>
+      <c r="D13" t="str">
+        <v>监听与转发配置</v>
+      </c>
+      <c r="E13" t="str">
+        <v>configure-backend</v>
+      </c>
+      <c r="F13" t="str">
+        <v>后端与服务器组</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B14" t="str">
+        <v>VPC功能使用咨询</v>
+      </c>
+      <c r="C14" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D14" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="E14" t="str">
+        <v>discover-intro</v>
+      </c>
+      <c r="F14" t="str">
+        <v>产品与能力咨询</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B15" t="str">
+        <v>VPC业务规则咨询</v>
+      </c>
+      <c r="C15" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D15" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="E15" t="str">
+        <v>discover-rules</v>
+      </c>
+      <c r="F15" t="str">
+        <v>业务规则与全局咨询</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B16" t="str">
+        <v>虚拟私有云业务规则咨询</v>
+      </c>
+      <c r="C16" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D16" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="E16" t="str">
+        <v>discover-rules</v>
+      </c>
+      <c r="F16" t="str">
+        <v>业务规则与全局咨询</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B17" t="str">
+        <v>全局流转</v>
+      </c>
+      <c r="C17" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D17" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="E17" t="str">
+        <v>discover-rules</v>
+      </c>
+      <c r="F17" t="str">
+        <v>业务规则与全局咨询</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B18" t="str">
+        <v>业务规则咨询/查询</v>
+      </c>
+      <c r="C18" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D18" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="E18" t="str">
+        <v>discover-rules</v>
+      </c>
+      <c r="F18" t="str">
+        <v>业务规则与全局咨询</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B19" t="str">
+        <v>VPC业务变更</v>
+      </c>
+      <c r="C19" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D19" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="E19" t="str">
+        <v>provision-subnet-change</v>
+      </c>
+      <c r="F19" t="str">
+        <v>变更网段与VPC业务变更</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B20" t="str">
+        <v>虚拟私有云业务变更</v>
+      </c>
+      <c r="C20" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D20" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="E20" t="str">
+        <v>provision-subnet-change</v>
+      </c>
+      <c r="F20" t="str">
+        <v>变更网段与VPC业务变更</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B21" t="str">
+        <v>VPCVPC删除修改操作问题</v>
+      </c>
+      <c r="C21" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D21" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="E21" t="str">
+        <v>provision-subnet-change</v>
+      </c>
+      <c r="F21" t="str">
+        <v>变更网段与VPC业务变更</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B22" t="str">
+        <v>VPC安装交付</v>
+      </c>
+      <c r="C22" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D22" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="E22" t="str">
+        <v>provision-delivery</v>
+      </c>
+      <c r="F22" t="str">
+        <v>安装交付与权限开通</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B23" t="str">
+        <v>虚拟私有云安装交付</v>
+      </c>
+      <c r="C23" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D23" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="E23" t="str">
+        <v>provision-delivery</v>
+      </c>
+      <c r="F23" t="str">
+        <v>安装交付与权限开通</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B24" t="str">
+        <v>VPC订购/开通</v>
+      </c>
+      <c r="C24" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D24" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="E24" t="str">
+        <v>provision-create</v>
+      </c>
+      <c r="F24" t="str">
+        <v>创建VPC与子网</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B25" t="str">
+        <v>VPC退订/取消</v>
+      </c>
+      <c r="C25" t="str">
+        <v>provision</v>
+      </c>
+      <c r="D25" t="str">
+        <v>创建与基础资源</v>
+      </c>
+      <c r="E25" t="str">
+        <v>provision-quota</v>
+      </c>
+      <c r="F25" t="str">
+        <v>配额与权限</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B26" t="str">
+        <v>VPC安全组配置异常、不生效</v>
+      </c>
+      <c r="C26" t="str">
+        <v>security</v>
+      </c>
+      <c r="D26" t="str">
+        <v>安全与访问控制</v>
+      </c>
+      <c r="E26" t="str">
+        <v>security-group</v>
+      </c>
+      <c r="F26" t="str">
+        <v>安全组配置与异常</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B27" t="str">
+        <v>VPCVPC下HAVIP无法使用问题</v>
+      </c>
+      <c r="C27" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D27" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="E27" t="str">
+        <v>operate-havip</v>
+      </c>
+      <c r="F27" t="str">
+        <v>HAVIP与高可用</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B28" t="str">
+        <v>云主机更换VPC</v>
+      </c>
+      <c r="C28" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D28" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="E28" t="str">
+        <v>operate-ecs</v>
+      </c>
+      <c r="F28" t="str">
+        <v>与云主机网卡联动</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B29" t="str">
+        <v>云主机内网问题-Linux系统主机内网异常</v>
+      </c>
+      <c r="C29" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D29" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="E29" t="str">
+        <v>operate-internal</v>
+      </c>
+      <c r="F29" t="str">
+        <v>内网互通异常</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B30" t="str">
+        <v>云主机外网连接-云主机DNS异常</v>
+      </c>
+      <c r="C30" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D30" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="E30" t="str">
+        <v>operate-ecs</v>
+      </c>
+      <c r="F30" t="str">
+        <v>与云主机网卡联动</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B31" t="str">
+        <v>云主机外网连接-linux系统主机无法连接外网</v>
+      </c>
+      <c r="C31" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D31" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="E31" t="str">
+        <v>operate-egress</v>
+      </c>
+      <c r="F31" t="str">
+        <v>出网与入网异常</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B32" t="str">
+        <v>云主机业务变更</v>
+      </c>
+      <c r="C32" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D32" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="E32" t="str">
+        <v>operate-ecs</v>
+      </c>
+      <c r="F32" t="str">
+        <v>与云主机网卡联动</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B33" t="str">
+        <v>产品咨询</v>
+      </c>
+      <c r="C33" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D33" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="E33" t="str">
+        <v>discover-intro</v>
+      </c>
+      <c r="F33" t="str">
+        <v>产品与能力咨询</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B34" t="str">
+        <v>产品功能</v>
+      </c>
+      <c r="C34" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D34" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="E34" t="str">
+        <v>discover-intro</v>
+      </c>
+      <c r="F34" t="str">
+        <v>产品与能力咨询</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B35" t="str">
+        <v>IP无法访问</v>
+      </c>
+      <c r="C35" t="str">
+        <v>operate</v>
+      </c>
+      <c r="D35" t="str">
+        <v>业务连通与运行</v>
+      </c>
+      <c r="E35" t="str">
+        <v>operate-egress</v>
+      </c>
+      <c r="F35" t="str">
+        <v>出网与入网异常</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>vpc</v>
+      </c>
+      <c r="B36" t="str">
+        <v>其他</v>
+      </c>
+      <c r="C36" t="str">
+        <v>discover</v>
+      </c>
+      <c r="D36" t="str">
+        <v>认知与组网规划</v>
+      </c>
+      <c r="E36" t="str">
+        <v>discover-intro</v>
+      </c>
+      <c r="F36" t="str">
+        <v>产品与能力咨询</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>eip</v>
+      </c>
+      <c r="B37" t="str">
+        <v>公网IP绑定/解绑失败</v>
+      </c>
+      <c r="C37" t="str">
+        <v>bind</v>
+      </c>
+      <c r="D37" t="str">
+        <v>绑定与网络配置</v>
+      </c>
+      <c r="E37" t="str">
+        <v>bind-resource</v>
+      </c>
+      <c r="F37" t="str">
+        <v>绑定/解绑云资源</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>问题类型名称</v>
-      </c>
-      <c r="B1" t="str">
-        <v>问题类型说明</v>
-      </c>
-      <c r="C1" t="str">
-        <v>参考关键词</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>可用性与连通性</v>
-      </c>
-      <c r="B2" t="str">
-        <v>服务达不到可用或连不通：中断、无法访问、大面积不可用</v>
-      </c>
-      <c r="C2" t="str">
-        <v>不通，无法访问，中断，不可用，连不上，502，503，504</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>性能与质量</v>
-      </c>
-      <c r="B3" t="str">
-        <v>能连上但质量差：慢、卡顿、延迟、丢包、抖动、超时</v>
-      </c>
-      <c r="C3" t="str">
-        <v>慢，卡顿，延迟，丢包，抖动，超时，不稳定，质量差</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>功能异常与缺陷</v>
-      </c>
-      <c r="B4" t="str">
-        <v>功能报错、结果不符预期、系统/底层异常，属缺陷或故障表现</v>
-      </c>
-      <c r="C4" t="str">
-        <v>报错，异常，失败，bug，不符合预期，底层异常，系统错误</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>功能需求与规划</v>
-      </c>
-      <c r="B5" t="str">
-        <v>用户希望新增或增强产品能力，属需求/建议，非现网故障</v>
-      </c>
-      <c r="C5" t="str">
-        <v>希望增加，建议，需求，缺少功能，不支持，增强</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>配置与对接</v>
-      </c>
-      <c r="B6" t="str">
-        <v>参数、绑定、路由、监听、白名单、跨产品对接等配置与集成问题</v>
-      </c>
-      <c r="C6" t="str">
-        <v>配置，绑定，解绑，路由，监听，策略，对接，参数，网卡，子网</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>资源与配额</v>
-      </c>
-      <c r="B7" t="str">
-        <v>开通失败、配额/容量/数量上限、权限不足、退订释放等资源生命周期与额度类</v>
-      </c>
-      <c r="C7" t="str">
-        <v>配额，上限，无法创建，开通失败，权限不足，退订，释放，删除，售罄</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>计费与商务</v>
-      </c>
-      <c r="B8" t="str">
-        <v>计费规则、账单金额、扣费逻辑、合同/折扣等商务计费域</v>
-      </c>
-      <c r="C8" t="str">
-        <v>计费，账单，扣费，资费，折扣，合同，商务</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>安全与合规</v>
-      </c>
-      <c r="B9" t="str">
-        <v>安全策略、攻击封堵、合规扫描、审计等安全合规域</v>
-      </c>
-      <c r="C9" t="str">
-        <v>安全，封堵，攻击，合规，审计，漏洞，风控，扫描</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>易用性体验</v>
-      </c>
-      <c r="B10" t="str">
-        <v>控制台、文档、流程难用；找不到入口、步骤冗长（非功能缺失、非服务投诉）</v>
-      </c>
-      <c r="C10" t="str">
-        <v>难用，文档，找不到，步骤复杂，不直观，体验，界面</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: request scene V2 — 9-class decision tree and taxonomy sync
Align request scene tagging with V2.0 rules (9 labels, priority tree, golden tests) and regenerate taxonomy config; document implementation and TAG-RS test plan.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/config/taxonomy/打标配置.xlsx
+++ b/public/config/taxonomy/打标配置.xlsx
@@ -6,9 +6,10 @@
     <sheet name="填写说明" sheetId="1" r:id="rId1"/>
     <sheet name="产品识别" sheetId="2" r:id="rId2"/>
     <sheet name="用户旅程" sheetId="3" r:id="rId3"/>
-    <sheet name="通用问题类型" sheetId="4" r:id="rId4"/>
-    <sheet name="请求节点-服务类型" sheetId="5" r:id="rId5"/>
-    <sheet name="请求节点-问题子类" sheetId="6" r:id="rId6"/>
+    <sheet name="请求场景" sheetId="4" r:id="rId4"/>
+    <sheet name="通用问题类型" sheetId="5" r:id="rId5"/>
+    <sheet name="请求节点-服务类型" sheetId="6" r:id="rId6"/>
+    <sheet name="请求节点-问题子类" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -402,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -462,105 +463,119 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>通用问题类型</v>
+        <v>请求场景</v>
       </c>
       <c r="B5" t="str">
         <v>全平台共用</v>
       </c>
       <c r="C5" t="str">
-        <v>无产品Key。问题类型名称、说明、参考关键词（12 类，与决策树 classifier 一致）</v>
+        <v>无产品Key。请求场景名称、说明、参考关键词（全产品共用，与问题类型同级）</v>
       </c>
       <c r="D5" t="str">
-        <v>可用性/连通性故障 | 业务完全中断、网络不通 | 不通,无法访问,中断</v>
+        <v>报障与排错 | 现网异常需排查恢复 | 故障,不通,异常</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>请求节点-服务类型</v>
+        <v>通用问题类型</v>
       </c>
       <c r="B6" t="str">
-        <v>可选；按产品Key</v>
+        <v>全平台共用</v>
       </c>
       <c r="C6" t="str">
-        <v>【弱参考·精确匹配】列「请求节点服务类型」须与工单路径第3段完全一致；一级ID/名称须存在于「用户旅程」。默认不用请求节点，仅设置中开启兜底且正文未识别时生效</v>
+        <v>无产品Key。问题类型名称、说明、参考关键词（12 类，与决策树 classifier 一致）</v>
       </c>
       <c r="D6" t="str">
-        <v>工单：请求节点：undefined--弹性公网IP--产品使用问题--公网IP绑定/解绑失败 → 第3段「产品使用问题」填本表</v>
+        <v>可用性/连通性故障 | 业务完全中断、网络不通 | 不通,无法访问,中断</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>请求节点-问题子类</v>
+        <v>请求节点-服务类型</v>
       </c>
       <c r="B7" t="str">
         <v>可选；按产品Key</v>
       </c>
       <c r="C7" t="str">
-        <v>【弱参考·精确匹配】列「请求节点问题子类」须与工单路径最后一段完全一致；二级ID 须为该一级下存在的环节</v>
+        <v>【弱参考·精确匹配】列「请求节点服务类型」须与工单路径第3段完全一致；一级ID/名称须存在于「用户旅程」。默认不用请求节点，仅设置中开启兜底且正文未识别时生效</v>
       </c>
       <c r="D7" t="str">
-        <v>同上工单 → 最后一段「公网IP绑定/解绑失败」填本表</v>
+        <v>工单：请求节点：undefined--弹性公网IP--产品使用问题--公网IP绑定/解绑失败 → 第3段「产品使用问题」填本表</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>（示例·路径拆分）</v>
+        <v>请求节点-问题子类</v>
       </c>
       <c r="B8" t="str">
-        <v>—</v>
+        <v>可选；按产品Key</v>
       </c>
       <c r="C8" t="str">
-        <v>请求节点：undefined--弹性公网IP--产品使用问题--公网IP绑定/解绑失败</v>
+        <v>【弱参考·精确匹配】列「请求节点问题子类」须与工单路径最后一段完全一致；二级ID 须为该一级下存在的环节</v>
       </c>
       <c r="D8" t="str">
-        <v>段1 undefined（忽略）| 段2 弹性公网IP（产品段）| 段3 产品使用问题→「请求节点-服务类型」| 段4 公网IP绑定/解绑失败→「请求节点-问题子类」</v>
+        <v>同上工单 → 最后一段「公网IP绑定/解绑失败」填本表</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>（示例·请求节点-服务类型）</v>
+        <v>（示例·路径拆分）</v>
       </c>
       <c r="B9" t="str">
-        <v>eip</v>
+        <v>—</v>
       </c>
       <c r="C9" t="str">
-        <v>产品Key | 请求节点服务类型 | 一级ID | 一级名称</v>
+        <v>请求节点：undefined--弹性公网IP--产品使用问题--公网IP绑定/解绑失败</v>
       </c>
       <c r="D9" t="str">
-        <v>eip | 产品使用问题 | operate | 日常运维与访问</v>
+        <v>段1 undefined（忽略）| 段2 弹性公网IP（产品段）| 段3 产品使用问题→「请求节点-服务类型」| 段4 公网IP绑定/解绑失败→「请求节点-问题子类」</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>（示例·请求节点-问题子类）</v>
+        <v>（示例·请求节点-服务类型）</v>
       </c>
       <c r="B10" t="str">
         <v>eip</v>
       </c>
       <c r="C10" t="str">
-        <v>产品Key | 请求节点问题子类 | 一级ID | 一级名称 | 二级ID | 二级名称</v>
+        <v>产品Key | 请求节点服务类型 | 一级ID | 一级名称</v>
       </c>
       <c r="D10" t="str">
-        <v>eip | 公网IP绑定/解绑失败 | bind | 绑定与网络配置 | bind-resource | 绑定/解绑云资源</v>
+        <v>eip | 产品使用问题 | operate | 日常运维与访问</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>（示例·请求节点-问题子类）</v>
+      </c>
+      <c r="B11" t="str">
+        <v>eip</v>
+      </c>
+      <c r="C11" t="str">
+        <v>产品Key | 请求节点问题子类 | 一级ID | 一级名称 | 二级ID | 二级名称</v>
+      </c>
+      <c r="D11" t="str">
+        <v>eip | 公网IP绑定/解绑失败 | bind | 绑定与网络配置 | bind-resource | 绑定/解绑云资源</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>（说明）</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B12" t="str">
         <v>—</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C12" t="str">
         <v>请求节点常不准确；主流程以处理意见/客户问题/LLM 为准。两表不做语义模糊匹配，只按原文对照</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D12" t="str">
         <v>—</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3455,6 +3470,127 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>请求场景名称</v>
+      </c>
+      <c r="B1" t="str">
+        <v>请求场景说明</v>
+      </c>
+      <c r="C1" t="str">
+        <v>参考关键词</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>报障与排错</v>
+      </c>
+      <c r="B2" t="str">
+        <v>现网业务已出现异常（中断、报错、性能劣化、安全事件等），客户请求技术排查与恢复</v>
+      </c>
+      <c r="C2" t="str">
+        <v>不通,掉线,中断,报错,崩溃,封堵,攻击,卡顿,慢,排查原因,抓包,解封,恢复,重启,无法访问,连接失败,超时,丢包,宕机,异常,故障,不可用,报障</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>资源操作申请</v>
+      </c>
+      <c r="B3" t="str">
+        <v>主动申请资源或权限的创建、变更、释放（含配额、权限、解售罄、轻载IP、灰度、扩容等），通常需要审批</v>
+      </c>
+      <c r="C3" t="str">
+        <v>申请,提升配额,扩容,增加IP,解售罄,轻载IP,灰度,解除8:1,开通权限,上架,申购,退订,释放,提升,配额,权限</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>操作指导</v>
+      </c>
+      <c r="B4" t="str">
+        <v>询问具体操作步骤、配置方法、最佳实践，无故障无异常，仅需指引</v>
+      </c>
+      <c r="C4" t="str">
+        <v>如何,怎么,怎样,操作步骤,配置方法,最佳实践,教程,设置,绑定,解绑,修改,步骤,方法</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>进度催办与协同</v>
+      </c>
+      <c r="B5" t="str">
+        <v>跟进已有订单/工单的进度，或请求云侧协助操作、协查、补充材料，核心是推动流程</v>
+      </c>
+      <c r="C5" t="str">
+        <v>催办,进度,查询订单,审批状态,建群,协查,补充材料,何时完成,帮忙跟进,协助处理,等了多久,还没好,处理到哪了</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>产品信息咨询</v>
+      </c>
+      <c r="B6" t="str">
+        <v>了解产品功能、规格、边界、价格、是否支持等认知信息，不要求立刻开通或排障</v>
+      </c>
+      <c r="C6" t="str">
+        <v>是否支持,规格,能力,功能说明,价格,多少钱,资费,区别,对比,支持,能不能,有什么功能,产品介绍,咨询</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>方案咨询与设计</v>
+      </c>
+      <c r="B7" t="str">
+        <v>需要架构设计、迁移/割接方案、组网规划等较复杂的业务方案支撑</v>
+      </c>
+      <c r="C7" t="str">
+        <v>方案,架构,选型,迁移,割接,落地,组网,规划,设计,跨区域,容灾,高可用</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>费用与账务</v>
+      </c>
+      <c r="B8" t="str">
+        <v>围绕账单、扣费、退款、发票、对账、资费核算的疑问或申诉</v>
+      </c>
+      <c r="C8" t="str">
+        <v>账单,扣费,退款,发票,对账,欠费,费用异常,多扣,少扣,怎么收费,计费规则,退费,冲销,出账</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>信息查询</v>
+      </c>
+      <c r="B9" t="str">
+        <v>纯粹查询状态、有效期、备案、资源归属等已有信息，无催办无操作</v>
+      </c>
+      <c r="C9" t="str">
+        <v>查有效期,查备案,查归属,查状态,是否还在,有没有,查询额度,核对信息</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>服务申诉与投诉</v>
+      </c>
+      <c r="B10" t="str">
+        <v>对客服态度、响应时效、处理流程不满，要求投诉、升级、回访</v>
+      </c>
+      <c r="C10" t="str">
+        <v>投诉,不满,态度差,升级处理,回访,响应慢,无人跟进,投诉到集团,要求赔偿,差评,服务太差</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C13"/>
   <sheetData>
     <row r="1">
@@ -3607,7 +3743,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D40"/>
   <sheetData>
@@ -4178,7 +4314,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F37"/>
   <sheetData>

</xml_diff>